<commit_message>
Mise a jour matrice de taches
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\audre\Documents\Github\Moteur-de-jeu-2D\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C713560F-51B9-405D-B8F7-BE4847BD04C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E2D6220-5FF0-4818-AB20-0289E5F908AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="49">
   <si>
     <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -148,6 +148,30 @@
   </si>
   <si>
     <t>Audrey / Elven</t>
+  </si>
+  <si>
+    <t>2.3 Calcule de la vitesse</t>
+  </si>
+  <si>
+    <t>15min</t>
+  </si>
+  <si>
+    <t>Réglage de problèmes de débugage</t>
+  </si>
+  <si>
+    <t>2.2 Équation différentielles question 1</t>
+  </si>
+  <si>
+    <t>2.1 Question 4</t>
+  </si>
+  <si>
+    <t>15 min</t>
+  </si>
+  <si>
+    <t>Le exel contenant la comparaison des résultats se trouve dans le git et est nommé "Comparaison_2.1.xlsx"</t>
+  </si>
+  <si>
+    <t>1h 15</t>
   </si>
 </sst>
 </file>
@@ -431,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" customWidth="1"/>
@@ -772,28 +796,97 @@
       <c r="E45" s="7"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
+      <c r="A46" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B46" s="5">
+        <v>46280</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
+      <c r="A47" s="2"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B48" s="7"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
-      <c r="E48" s="7"/>
-    </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B49" s="7"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
+      <c r="B48" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B49" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="E49" s="7"/>
+    </row>
+    <row r="50" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B50" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E50" s="7"/>
+    </row>
+    <row r="51" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B51" t="s">
+        <v>45</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B52" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E52" s="7"/>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B55" s="7"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.70069444444444495" right="0.70069444444444495" top="0.75208333333333299" bottom="0.75208333333333299" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
rotation et remplacement de l'image du joueur
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="56">
   <si>
     <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
   </si>
@@ -169,6 +169,9 @@
     <t xml:space="preserve">2.2 Équation différentielles question 1 à 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Séances :</t>
+  </si>
+  <si>
     <t xml:space="preserve">2.2 Équation différentielles question 4 à 6</t>
   </si>
   <si>
@@ -176,6 +179,15 @@
   </si>
   <si>
     <t xml:space="preserve">2.3 fin des calculs et courbes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 début affichage image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fin affichage image et rotation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aide ia pour le sprite qui etait de taille 0*0 avec une texture de la bonne taille</t>
   </si>
 </sst>
 </file>
@@ -283,44 +295,48 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -513,480 +529,530 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="31.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="9.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="31.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="9.11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
+      <c r="A4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="G7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="G7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C8" s="5"/>
-      <c r="G8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="G8" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="5"/>
+      <c r="G13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G14" s="5"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="7" t="n">
         <v>46274</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
+      <c r="A21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="D23" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E23" s="8"/>
+      <c r="E23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E24" s="8"/>
+      <c r="E24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E25" s="8"/>
+      <c r="E25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E26" s="4"/>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B30" s="7" t="n">
         <v>46275</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2"/>
+      <c r="A31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E33" s="8"/>
+      <c r="E33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="8" t="s">
+      <c r="B34" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="D34" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E34" s="8"/>
+      <c r="E34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D35" s="8" t="s">
+      <c r="D35" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E35" s="8"/>
+      <c r="E35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D36" s="8" t="s">
+      <c r="D36" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E36" s="8"/>
+      <c r="E36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D37" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
+      <c r="A39" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B39" s="6" t="n">
+      <c r="B39" s="7" t="n">
         <v>46279</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2"/>
+      <c r="A40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="D41" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="9" t="s">
+      <c r="B42" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D42" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E42" s="9" t="s">
+      <c r="E42" s="10" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="9" t="s">
+      <c r="B43" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="E43" s="9" t="s">
+      <c r="E43" s="10" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="C44" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D44" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E44" s="8"/>
+      <c r="E44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2" t="s">
+      <c r="A46" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="6" t="n">
+      <c r="B46" s="7" t="n">
         <v>46280</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2"/>
+      <c r="A47" s="3"/>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C48" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="D48" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="E48" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="C49" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D49" s="8" t="s">
+      <c r="D49" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E49" s="8" t="s">
+      <c r="E49" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C50" s="8" t="s">
+      <c r="C50" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D50" s="8" t="s">
+      <c r="D50" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E50" s="8"/>
+      <c r="E50" s="9"/>
     </row>
     <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="0" t="s">
+      <c r="B51" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C51" s="8" t="s">
+      <c r="C51" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D51" s="8" t="s">
+      <c r="D51" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="8" t="s">
+      <c r="E51" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B52" s="8" t="s">
+      <c r="B52" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C52" s="8" t="s">
+      <c r="C52" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D52" s="8" t="s">
+      <c r="D52" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E52" s="8"/>
+      <c r="E52" s="9"/>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="8"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="8"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="9"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="8"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="8"/>
-      <c r="E54" s="8"/>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2" t="s">
+      <c r="A55" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B55" s="7" t="n">
+        <v>46282</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3"/>
+    </row>
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B55" s="6" t="n">
-        <v>46282</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="2"/>
-    </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="2" t="s">
+      <c r="B64" s="7" t="n">
+        <v>46283</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="3"/>
+    </row>
+    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="C66" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="D66" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E57" s="2" t="s">
+      <c r="E66" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="C58" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="D58" s="0" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="0" t="s">
-        <v>51</v>
-      </c>
-      <c r="C59" s="0" t="s">
+    <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C67" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D59" s="0" t="s">
-        <v>50</v>
+      <c r="D67" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E67" s="9" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mise a jour de la matrice des taches
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -1,21 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\audre\Documents\Github\Moteur-de-jeu-2D\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D4EB483-DE27-433B-938F-82432833A8D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="7"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuille1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -25,224 +20,251 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="59">
-  <si>
-    <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
-  </si>
-  <si>
-    <t>Séance :</t>
-  </si>
-  <si>
-    <t>XX/XX/XXXX</t>
-  </si>
-  <si>
-    <t>Tâche</t>
-  </si>
-  <si>
-    <t>Etudiant</t>
-  </si>
-  <si>
-    <t>Charge retenue (h)</t>
-  </si>
-  <si>
-    <t>Commentaires</t>
-  </si>
-  <si>
-    <t>Attention :</t>
-  </si>
-  <si>
-    <t>1. Seules les tâches techniques sont à inscrire (maths, code, ...).</t>
-  </si>
-  <si>
-    <t>2. Les tâches autres (gestion, mise en page, ...) seront valorisées à une charge de 0 heure.</t>
-  </si>
-  <si>
-    <t>3. Les tâches réalisées avec une IA doivent faire apparaître IA dans la colonne Etudiant. Elles ne sont pas prises en compte pour la répartition de la charge.</t>
-  </si>
-  <si>
-    <t>4. La colonne 'Charge retenue' contient le temps approximatif. Maximum de 2 heures par étudiant et par séance.</t>
-  </si>
-  <si>
-    <t>5. La répartition individuelle est calculée sur la base des heures individuelles retenues et la somme des heures totales retenues.</t>
-  </si>
-  <si>
-    <t>6. Cette matrice doit être remplie par le groupe et la répartition indiquée être validée par tout le groupe.</t>
-  </si>
-  <si>
-    <t>7. Les contributions indiquées doivent refléter l'apport au projet, non le nombre d'heures devant l'écran.</t>
-  </si>
-  <si>
-    <t>Réponse aux questions du 1.2</t>
-  </si>
-  <si>
-    <t>Audrey</t>
-  </si>
-  <si>
-    <t>20 min</t>
-  </si>
-  <si>
-    <t>Configuration du git</t>
-  </si>
-  <si>
-    <t>Elven</t>
-  </si>
-  <si>
-    <t>10 min</t>
-  </si>
-  <si>
-    <t>Mise en place du projet avec SFML</t>
-  </si>
-  <si>
-    <t>1h 30</t>
-  </si>
-  <si>
-    <t>Alizee</t>
-  </si>
-  <si>
-    <t>30min</t>
-  </si>
-  <si>
-    <t>Correction pour passer de sfml 2 a 3</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="61">
+  <si>
+    <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Séance :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XX/XX/XXXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tâche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etudiant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charge retenue (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commentaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attention :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Seules les tâches techniques sont à inscrire (maths, code, ...).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Les tâches autres (gestion, mise en page, ...) seront valorisées à une charge de 0 heure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Les tâches réalisées avec une IA doivent faire apparaître IA dans la colonne Etudiant. Elles ne sont pas prises en compte pour la répartition de la charge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. La colonne 'Charge retenue' contient le temps approximatif. Maximum de 2 heures par étudiant et par séance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. La répartition individuelle est calculée sur la base des heures individuelles retenues et la somme des heures totales retenues.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Cette matrice doit être remplie par le groupe et la répartition indiquée être validée par tout le groupe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Les contributions indiquées doivent refléter l'apport au projet, non le nombre d'heures devant l'écran.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réponse aux questions du 1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration du git</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place du projet avec SFML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1h 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alizee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correction pour passer de sfml 2 a 3</t>
   </si>
   <si>
     <t xml:space="preserve">30min </t>
   </si>
   <si>
-    <t>Code 1,2 conversion</t>
-  </si>
-  <si>
-    <t>Code 1,2 debug</t>
-  </si>
-  <si>
-    <t>1h</t>
-  </si>
-  <si>
-    <t>Formule 1,2</t>
-  </si>
-  <si>
-    <t>Questions 1.2</t>
-  </si>
-  <si>
-    <t>30 min</t>
-  </si>
-  <si>
-    <t>déplacement v1 simple</t>
-  </si>
-  <si>
-    <t>Alizée</t>
-  </si>
-  <si>
-    <t>code et question correspondante</t>
-  </si>
-  <si>
-    <t>déplacement v2 diagonal</t>
+    <t xml:space="preserve">Code 1,2 conversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code 1,2 debug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formule 1,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Questions 1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">déplacement v1 simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alizée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">code et question correspondante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">déplacement v2 diagonal</t>
   </si>
   <si>
     <t xml:space="preserve">Alizée </t>
   </si>
   <si>
-    <t>code et questions correspondantes</t>
-  </si>
-  <si>
-    <t>2.1 Questions 1 à 3</t>
-  </si>
-  <si>
-    <t>Audrey / Elven</t>
-  </si>
-  <si>
-    <t>2.3</t>
-  </si>
-  <si>
-    <t>45min</t>
-  </si>
-  <si>
-    <t>Calcul de la vitesse et affichage en debug, ajout d’un txt pour la police d’écriture et debut question</t>
-  </si>
-  <si>
-    <t>Réglage de problèmes de débug et release</t>
-  </si>
-  <si>
-    <t>2.1 Question 4</t>
-  </si>
-  <si>
-    <t>15 min</t>
-  </si>
-  <si>
-    <t>Le exel contenant la comparaison des résultats se trouve dans le git et est nommé "Courbes_exercices.xlsx"</t>
-  </si>
-  <si>
-    <t>2.2 Équation différentielles question 1 à 3</t>
-  </si>
-  <si>
-    <t>Séances :</t>
-  </si>
-  <si>
-    <t>2.2 Équation différentielles question 4 à 6</t>
-  </si>
-  <si>
-    <t>1h30</t>
+    <t xml:space="preserve">code et questions correspondantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Questions 1 à 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audrey / Elven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcul de la vitesse et affichage en debug, ajout d’un txt pour la police d’écriture et debut question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réglage de problèmes de débug et release</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Question 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le exel contenant la comparaison des résultats se trouve dans le git et est nommé "Courbes_exercices.xlsx"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 Équation différentielles question 1 à 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Séances :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 Équation différentielles question 4 à 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1h30</t>
   </si>
   <si>
     <t xml:space="preserve">2.3 fin des calculs et courbes </t>
   </si>
   <si>
-    <t>5 début affichage image</t>
-  </si>
-  <si>
-    <t>Fin affichage image et rotation</t>
-  </si>
-  <si>
-    <t>Aide ia pour le sprite qui etait de taille 0*0 avec une texture de la bonne taille</t>
-  </si>
-  <si>
-    <t>6.1 Ajout d’autres entités</t>
-  </si>
-  <si>
-    <t>2h</t>
-  </si>
-  <si>
-    <t>aide IA pour la structuration de la classe abstraîte Entity puis modification et restructurationdu code pour le débugage</t>
+    <t xml:space="preserve">5 début affichage image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fin affichage image et rotation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aide ia pour le sprite qui etait de taille 0*0 avec une texture de la bonne taille</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.1 Ajout d’autres entités</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aide IA pour la structuration de la classe abstraîte Entity puis modification et restructurationdu code pour le débugage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 ajout cadre et rebond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 modification rebond et energie</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
-      <u/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <u val="single"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -255,7 +277,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -263,46 +285,82 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="New Office">
       <a:dk1>
@@ -344,14 +402,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1"/>
+        <a:ea typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:cs typeface="Arial" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:ea typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:cs typeface="Arial" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -381,7 +439,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -405,7 +463,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -465,46 +523,47 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:G83"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
-    <col min="2" max="2" width="24.21875" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" customWidth="1"/>
-    <col min="5" max="5" width="31.88671875" customWidth="1"/>
-    <col min="6" max="8" width="9.109375" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="31.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="9.11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="0" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
@@ -518,77 +577,77 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="4"/>
       <c r="G8" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="0" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="0" t="s">
         <v>9</v>
       </c>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0" t="s">
         <v>10</v>
       </c>
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="0" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="5" t="n">
         <v>46274</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
         <v>3</v>
       </c>
@@ -602,7 +661,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="7" t="s">
         <v>15</v>
       </c>
@@ -614,7 +673,7 @@
       </c>
       <c r="E23" s="7"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="7" t="s">
         <v>18</v>
       </c>
@@ -626,7 +685,7 @@
       </c>
       <c r="E24" s="7"/>
     </row>
-    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
         <v>21</v>
       </c>
@@ -638,7 +697,7 @@
       </c>
       <c r="E25" s="7"/>
     </row>
-    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="7" t="s">
         <v>15</v>
       </c>
@@ -650,30 +709,30 @@
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B30" s="5">
+      <c r="B30" s="5" t="n">
         <v>46275</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
         <v>3</v>
       </c>
@@ -687,7 +746,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="7" t="s">
         <v>25</v>
       </c>
@@ -699,7 +758,7 @@
       </c>
       <c r="E33" s="7"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="7" t="s">
         <v>27</v>
       </c>
@@ -711,7 +770,7 @@
       </c>
       <c r="E34" s="7"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="7" t="s">
         <v>28</v>
       </c>
@@ -723,7 +782,7 @@
       </c>
       <c r="E35" s="7"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="7" t="s">
         <v>30</v>
       </c>
@@ -735,7 +794,7 @@
       </c>
       <c r="E36" s="7"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="7" t="s">
         <v>31</v>
       </c>
@@ -746,18 +805,18 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B39" s="5">
+      <c r="B39" s="5" t="n">
         <v>46279</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="2" t="s">
         <v>3</v>
       </c>
@@ -771,7 +830,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="8" t="s">
         <v>33</v>
       </c>
@@ -785,7 +844,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="s">
         <v>36</v>
       </c>
@@ -799,7 +858,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="7" t="s">
         <v>39</v>
       </c>
@@ -811,24 +870,24 @@
       </c>
       <c r="E44" s="7"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
       <c r="E45" s="7"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="5">
+      <c r="B46" s="5" t="n">
         <v>46280</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="2" t="s">
         <v>3</v>
       </c>
@@ -842,7 +901,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="7" t="s">
         <v>41</v>
       </c>
@@ -856,7 +915,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="7" t="s">
         <v>44</v>
       </c>
@@ -868,8 +927,8 @@
       </c>
       <c r="E50" s="7"/>
     </row>
-    <row r="51" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B51" t="s">
+    <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="0" t="s">
         <v>45</v>
       </c>
       <c r="C51" s="7" t="s">
@@ -882,7 +941,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="7" t="s">
         <v>48</v>
       </c>
@@ -894,30 +953,30 @@
       </c>
       <c r="E52" s="7"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B55" s="5">
+      <c r="B55" s="5" t="n">
         <v>46282</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="2" t="s">
         <v>3</v>
       </c>
@@ -931,51 +990,51 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B58" t="s">
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D58" s="0" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B59" t="s">
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C59" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D59" s="0" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B60" t="s">
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D60" s="0" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B64" s="5">
+      <c r="B64" s="5" t="n">
         <v>46283</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
         <v>3</v>
       </c>
@@ -989,7 +1048,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="7" t="s">
         <v>54</v>
       </c>
@@ -1003,7 +1062,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="68" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="7" t="s">
         <v>56</v>
       </c>
@@ -1014,21 +1073,21 @@
         <v>29</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B70" s="5">
+      <c r="B70" s="5" t="n">
         <v>46286</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="6" t="s">
         <v>3</v>
       </c>
@@ -1042,7 +1101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="7" t="s">
         <v>56</v>
       </c>
@@ -1050,72 +1109,96 @@
         <v>16</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E73" s="7"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B74" s="7"/>
-      <c r="C74" s="7"/>
-      <c r="D74" s="7"/>
+    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B74" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D74" s="7" t="s">
+        <v>58</v>
+      </c>
       <c r="E74" s="7"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="7"/>
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
       <c r="E75" s="7"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="7"/>
       <c r="C76" s="7"/>
       <c r="D76" s="7"/>
       <c r="E76" s="7"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B77" s="7"/>
-      <c r="C77" s="7"/>
-      <c r="D77" s="7"/>
-      <c r="E77" s="7"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B78" s="7"/>
-      <c r="C78" s="7"/>
-      <c r="D78" s="7"/>
-      <c r="E78" s="7"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B79" s="7"/>
-      <c r="C79" s="7"/>
-      <c r="D79" s="7"/>
-      <c r="E79" s="7"/>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B80" s="7"/>
-      <c r="C80" s="7"/>
-      <c r="D80" s="7"/>
+    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B77" s="5" t="n">
+        <v>46287</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="2"/>
+    </row>
+    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B79" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>58</v>
+      </c>
       <c r="E80" s="7"/>
     </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="7"/>
       <c r="C81" s="7"/>
       <c r="D81" s="7"/>
       <c r="E81" s="7"/>
     </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="7"/>
       <c r="C82" s="7"/>
       <c r="D82" s="7"/>
       <c r="E82" s="7"/>
     </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="7"/>
       <c r="C83" s="7"/>
       <c r="D83" s="7"/>
       <c r="E83" s="7"/>
     </row>
   </sheetData>
-  <pageMargins left="0.70069444444444495" right="0.70069444444444495" top="0.75208333333333299" bottom="0.75208333333333299" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.700694444444445" right="0.700694444444445" top="0.752083333333333" bottom="0.752083333333333" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mise a jour du suivi pero et du tableau de tache
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="7"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\audre\Documents\Github\Moteur-de-jeu-2D\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42E7181-A746-46A1-A929-2BE2176489E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Feuille1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -20,251 +25,233 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="61">
-  <si>
-    <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Séance :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XX/XX/XXXX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tâche</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Etudiant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charge retenue (h)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commentaires</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attention :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Seules les tâches techniques sont à inscrire (maths, code, ...).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Les tâches autres (gestion, mise en page, ...) seront valorisées à une charge de 0 heure.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Les tâches réalisées avec une IA doivent faire apparaître IA dans la colonne Etudiant. Elles ne sont pas prises en compte pour la répartition de la charge.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. La colonne 'Charge retenue' contient le temps approximatif. Maximum de 2 heures par étudiant et par séance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. La répartition individuelle est calculée sur la base des heures individuelles retenues et la somme des heures totales retenues.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Cette matrice doit être remplie par le groupe et la répartition indiquée être validée par tout le groupe.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Les contributions indiquées doivent refléter l'apport au projet, non le nombre d'heures devant l'écran.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réponse aux questions du 1.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audrey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configuration du git</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elven</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mise en place du projet avec SFML</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1h 30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alizee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Correction pour passer de sfml 2 a 3</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="62">
+  <si>
+    <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
+  </si>
+  <si>
+    <t>Séance :</t>
+  </si>
+  <si>
+    <t>XX/XX/XXXX</t>
+  </si>
+  <si>
+    <t>Tâche</t>
+  </si>
+  <si>
+    <t>Etudiant</t>
+  </si>
+  <si>
+    <t>Charge retenue (h)</t>
+  </si>
+  <si>
+    <t>Commentaires</t>
+  </si>
+  <si>
+    <t>Attention :</t>
+  </si>
+  <si>
+    <t>1. Seules les tâches techniques sont à inscrire (maths, code, ...).</t>
+  </si>
+  <si>
+    <t>2. Les tâches autres (gestion, mise en page, ...) seront valorisées à une charge de 0 heure.</t>
+  </si>
+  <si>
+    <t>3. Les tâches réalisées avec une IA doivent faire apparaître IA dans la colonne Etudiant. Elles ne sont pas prises en compte pour la répartition de la charge.</t>
+  </si>
+  <si>
+    <t>4. La colonne 'Charge retenue' contient le temps approximatif. Maximum de 2 heures par étudiant et par séance.</t>
+  </si>
+  <si>
+    <t>5. La répartition individuelle est calculée sur la base des heures individuelles retenues et la somme des heures totales retenues.</t>
+  </si>
+  <si>
+    <t>6. Cette matrice doit être remplie par le groupe et la répartition indiquée être validée par tout le groupe.</t>
+  </si>
+  <si>
+    <t>7. Les contributions indiquées doivent refléter l'apport au projet, non le nombre d'heures devant l'écran.</t>
+  </si>
+  <si>
+    <t>Réponse aux questions du 1.2</t>
+  </si>
+  <si>
+    <t>Audrey</t>
+  </si>
+  <si>
+    <t>20 min</t>
+  </si>
+  <si>
+    <t>Configuration du git</t>
+  </si>
+  <si>
+    <t>Elven</t>
+  </si>
+  <si>
+    <t>10 min</t>
+  </si>
+  <si>
+    <t>Mise en place du projet avec SFML</t>
+  </si>
+  <si>
+    <t>1h 30</t>
+  </si>
+  <si>
+    <t>Alizee</t>
+  </si>
+  <si>
+    <t>30min</t>
+  </si>
+  <si>
+    <t>Correction pour passer de sfml 2 a 3</t>
   </si>
   <si>
     <t xml:space="preserve">30min </t>
   </si>
   <si>
-    <t xml:space="preserve">Code 1,2 conversion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code 1,2 debug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formule 1,2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Questions 1.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30 min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">déplacement v1 simple</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alizée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">code et question correspondante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">déplacement v2 diagonal</t>
+    <t>Code 1,2 conversion</t>
+  </si>
+  <si>
+    <t>Code 1,2 debug</t>
+  </si>
+  <si>
+    <t>1h</t>
+  </si>
+  <si>
+    <t>Formule 1,2</t>
+  </si>
+  <si>
+    <t>Questions 1.2</t>
+  </si>
+  <si>
+    <t>30 min</t>
+  </si>
+  <si>
+    <t>déplacement v1 simple</t>
+  </si>
+  <si>
+    <t>Alizée</t>
+  </si>
+  <si>
+    <t>code et question correspondante</t>
+  </si>
+  <si>
+    <t>déplacement v2 diagonal</t>
   </si>
   <si>
     <t xml:space="preserve">Alizée </t>
   </si>
   <si>
-    <t xml:space="preserve">code et questions correspondantes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1 Questions 1 à 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audrey / Elven</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calcul de la vitesse et affichage en debug, ajout d’un txt pour la police d’écriture et debut question</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réglage de problèmes de débug et release</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1 Question 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le exel contenant la comparaison des résultats se trouve dans le git et est nommé "Courbes_exercices.xlsx"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2 Équation différentielles question 1 à 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Séances :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2 Équation différentielles question 4 à 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1h30</t>
+    <t>code et questions correspondantes</t>
+  </si>
+  <si>
+    <t>2.1 Questions 1 à 3</t>
+  </si>
+  <si>
+    <t>Audrey / Elven</t>
+  </si>
+  <si>
+    <t>2.3</t>
+  </si>
+  <si>
+    <t>45min</t>
+  </si>
+  <si>
+    <t>Calcul de la vitesse et affichage en debug, ajout d’un txt pour la police d’écriture et debut question</t>
+  </si>
+  <si>
+    <t>Réglage de problèmes de débug et release</t>
+  </si>
+  <si>
+    <t>2.1 Question 4</t>
+  </si>
+  <si>
+    <t>15 min</t>
+  </si>
+  <si>
+    <t>Le exel contenant la comparaison des résultats se trouve dans le git et est nommé "Courbes_exercices.xlsx"</t>
+  </si>
+  <si>
+    <t>2.2 Équation différentielles question 1 à 3</t>
+  </si>
+  <si>
+    <t>Séances :</t>
+  </si>
+  <si>
+    <t>2.2 Équation différentielles question 4 à 6</t>
+  </si>
+  <si>
+    <t>1h30</t>
   </si>
   <si>
     <t xml:space="preserve">2.3 fin des calculs et courbes </t>
   </si>
   <si>
-    <t xml:space="preserve">5 début affichage image</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fin affichage image et rotation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aide ia pour le sprite qui etait de taille 0*0 avec une texture de la bonne taille</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.1 Ajout d’autres entités</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aide IA pour la structuration de la classe abstraîte Entity puis modification et restructurationdu code pour le débugage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 ajout cadre et rebond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 modification rebond et energie</t>
+    <t>5 début affichage image</t>
+  </si>
+  <si>
+    <t>Fin affichage image et rotation</t>
+  </si>
+  <si>
+    <t>Aide ia pour le sprite qui etait de taille 0*0 avec une texture de la bonne taille</t>
+  </si>
+  <si>
+    <t>6.1 Ajout d’autres entités</t>
+  </si>
+  <si>
+    <t>aide IA pour la structuration de la classe abstraîte Entity puis modification et restructurationdu code pour le débugage</t>
+  </si>
+  <si>
+    <t>2h</t>
+  </si>
+  <si>
+    <t>5 ajout cadre et rebond</t>
+  </si>
+  <si>
+    <t>5 modification rebond et energie</t>
+  </si>
+  <si>
+    <t>refactorisation debug</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <u val="single"/>
+      <b/>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -277,7 +264,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -285,82 +272,46 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="New Office">
       <a:dk1>
@@ -402,14 +353,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1"/>
-        <a:ea typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:cs typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:cs typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -439,7 +390,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -463,7 +414,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -523,47 +474,46 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G83"/>
-  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="31.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="9.11"/>
+    <col min="1" max="1" width="9.109375" customWidth="1"/>
+    <col min="2" max="2" width="24.21875" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" customWidth="1"/>
+    <col min="5" max="5" width="31.88671875" customWidth="1"/>
+    <col min="6" max="8" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
@@ -577,77 +527,77 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C8" s="4"/>
       <c r="G8" s="4"/>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
         <v>9</v>
       </c>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
         <v>10</v>
       </c>
       <c r="G14" s="4"/>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0" t="s">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0" t="s">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B20" s="5">
         <v>46274</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B22" s="6" t="s">
         <v>3</v>
       </c>
@@ -661,7 +611,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B23" s="7" t="s">
         <v>15</v>
       </c>
@@ -673,7 +623,7 @@
       </c>
       <c r="E23" s="7"/>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B24" s="7" t="s">
         <v>18</v>
       </c>
@@ -685,7 +635,7 @@
       </c>
       <c r="E24" s="7"/>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B25" s="7" t="s">
         <v>21</v>
       </c>
@@ -697,7 +647,7 @@
       </c>
       <c r="E25" s="7"/>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B26" s="7" t="s">
         <v>15</v>
       </c>
@@ -709,30 +659,30 @@
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
     </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B30" s="5" t="n">
+      <c r="B30" s="5">
         <v>46275</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B32" s="2" t="s">
         <v>3</v>
       </c>
@@ -746,7 +696,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B33" s="7" t="s">
         <v>25</v>
       </c>
@@ -758,7 +708,7 @@
       </c>
       <c r="E33" s="7"/>
     </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B34" s="7" t="s">
         <v>27</v>
       </c>
@@ -770,7 +720,7 @@
       </c>
       <c r="E34" s="7"/>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B35" s="7" t="s">
         <v>28</v>
       </c>
@@ -782,7 +732,7 @@
       </c>
       <c r="E35" s="7"/>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B36" s="7" t="s">
         <v>30</v>
       </c>
@@ -794,7 +744,7 @@
       </c>
       <c r="E36" s="7"/>
     </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B37" s="7" t="s">
         <v>31</v>
       </c>
@@ -805,18 +755,18 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B39" s="5" t="n">
+      <c r="B39" s="5">
         <v>46279</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B41" s="2" t="s">
         <v>3</v>
       </c>
@@ -830,7 +780,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B42" s="8" t="s">
         <v>33</v>
       </c>
@@ -844,7 +794,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B43" s="8" t="s">
         <v>36</v>
       </c>
@@ -858,7 +808,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B44" s="7" t="s">
         <v>39</v>
       </c>
@@ -870,24 +820,24 @@
       </c>
       <c r="E44" s="7"/>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
       <c r="E45" s="7"/>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="5" t="n">
+      <c r="B46" s="5">
         <v>46280</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="2"/>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B48" s="2" t="s">
         <v>3</v>
       </c>
@@ -901,7 +851,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B49" s="7" t="s">
         <v>41</v>
       </c>
@@ -915,7 +865,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B50" s="7" t="s">
         <v>44</v>
       </c>
@@ -927,8 +877,8 @@
       </c>
       <c r="E50" s="7"/>
     </row>
-    <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="0" t="s">
+    <row r="51" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B51" t="s">
         <v>45</v>
       </c>
       <c r="C51" s="7" t="s">
@@ -941,7 +891,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B52" s="7" t="s">
         <v>48</v>
       </c>
@@ -953,30 +903,30 @@
       </c>
       <c r="E52" s="7"/>
     </row>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
     </row>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
     </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B55" s="5" t="n">
+      <c r="B55" s="5">
         <v>46282</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B57" s="2" t="s">
         <v>3</v>
       </c>
@@ -990,51 +940,51 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B58" s="0" t="s">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B58" t="s">
         <v>50</v>
       </c>
-      <c r="C58" s="0" t="s">
+      <c r="C58" t="s">
         <v>40</v>
       </c>
-      <c r="D58" s="0" t="s">
+      <c r="D58" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="0" t="s">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B59" t="s">
         <v>52</v>
       </c>
-      <c r="C59" s="0" t="s">
+      <c r="C59" t="s">
         <v>34</v>
       </c>
-      <c r="D59" s="0" t="s">
+      <c r="D59" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="0" t="s">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B60" t="s">
         <v>53</v>
       </c>
-      <c r="C60" s="0" t="s">
+      <c r="C60" t="s">
         <v>34</v>
       </c>
-      <c r="D60" s="0" t="s">
+      <c r="D60" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B64" s="5" t="n">
+      <c r="B64" s="5">
         <v>46283</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="2"/>
     </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B66" s="6" t="s">
         <v>3</v>
       </c>
@@ -1048,7 +998,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B67" s="7" t="s">
         <v>54</v>
       </c>
@@ -1062,7 +1012,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B68" s="7" t="s">
         <v>56</v>
       </c>
@@ -1076,18 +1026,18 @@
         <v>57</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B70" s="5" t="n">
+      <c r="B70" s="5">
         <v>46286</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="2"/>
     </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B72" s="6" t="s">
         <v>3</v>
       </c>
@@ -1101,7 +1051,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B73" s="7" t="s">
         <v>56</v>
       </c>
@@ -1113,7 +1063,7 @@
       </c>
       <c r="E73" s="7"/>
     </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B74" s="7" t="s">
         <v>59</v>
       </c>
@@ -1125,30 +1075,30 @@
       </c>
       <c r="E74" s="7"/>
     </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B75" s="7"/>
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
       <c r="E75" s="7"/>
     </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B76" s="7"/>
       <c r="C76" s="7"/>
       <c r="D76" s="7"/>
       <c r="E76" s="7"/>
     </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B77" s="5" t="n">
+      <c r="B77" s="5">
         <v>46287</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
     </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B79" s="6" t="s">
         <v>3</v>
       </c>
@@ -1162,7 +1112,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B80" s="7" t="s">
         <v>60</v>
       </c>
@@ -1174,31 +1124,32 @@
       </c>
       <c r="E80" s="7"/>
     </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B81" s="7"/>
-      <c r="C81" s="7"/>
-      <c r="D81" s="7"/>
+    <row r="81" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B81" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>58</v>
+      </c>
       <c r="E81" s="7"/>
     </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B82" s="7"/>
       <c r="C82" s="7"/>
       <c r="D82" s="7"/>
       <c r="E82" s="7"/>
     </row>
-    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B83" s="7"/>
       <c r="C83" s="7"/>
       <c r="D83" s="7"/>
       <c r="E83" s="7"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.700694444444445" right="0.700694444444445" top="0.752083333333333" bottom="0.752083333333333" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageMargins left="0.70069444444444495" right="0.70069444444444495" top="0.75208333333333299" bottom="0.75208333333333299" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
mise a jour matrice des taches
</commit_message>
<xml_diff>
--- a/Matrice des tâches.xlsx
+++ b/Matrice des tâches.xlsx
@@ -1,21 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\audre\Documents\Github\Moteur-de-jeu-2D\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42E7181-A746-46A1-A929-2BE2176489E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="7"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuille1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -25,233 +20,263 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="62">
-  <si>
-    <t>Matrice de répartition de charges (à remplir à chaque séance)</t>
-  </si>
-  <si>
-    <t>Séance :</t>
-  </si>
-  <si>
-    <t>XX/XX/XXXX</t>
-  </si>
-  <si>
-    <t>Tâche</t>
-  </si>
-  <si>
-    <t>Etudiant</t>
-  </si>
-  <si>
-    <t>Charge retenue (h)</t>
-  </si>
-  <si>
-    <t>Commentaires</t>
-  </si>
-  <si>
-    <t>Attention :</t>
-  </si>
-  <si>
-    <t>1. Seules les tâches techniques sont à inscrire (maths, code, ...).</t>
-  </si>
-  <si>
-    <t>2. Les tâches autres (gestion, mise en page, ...) seront valorisées à une charge de 0 heure.</t>
-  </si>
-  <si>
-    <t>3. Les tâches réalisées avec une IA doivent faire apparaître IA dans la colonne Etudiant. Elles ne sont pas prises en compte pour la répartition de la charge.</t>
-  </si>
-  <si>
-    <t>4. La colonne 'Charge retenue' contient le temps approximatif. Maximum de 2 heures par étudiant et par séance.</t>
-  </si>
-  <si>
-    <t>5. La répartition individuelle est calculée sur la base des heures individuelles retenues et la somme des heures totales retenues.</t>
-  </si>
-  <si>
-    <t>6. Cette matrice doit être remplie par le groupe et la répartition indiquée être validée par tout le groupe.</t>
-  </si>
-  <si>
-    <t>7. Les contributions indiquées doivent refléter l'apport au projet, non le nombre d'heures devant l'écran.</t>
-  </si>
-  <si>
-    <t>Réponse aux questions du 1.2</t>
-  </si>
-  <si>
-    <t>Audrey</t>
-  </si>
-  <si>
-    <t>20 min</t>
-  </si>
-  <si>
-    <t>Configuration du git</t>
-  </si>
-  <si>
-    <t>Elven</t>
-  </si>
-  <si>
-    <t>10 min</t>
-  </si>
-  <si>
-    <t>Mise en place du projet avec SFML</t>
-  </si>
-  <si>
-    <t>1h 30</t>
-  </si>
-  <si>
-    <t>Alizee</t>
-  </si>
-  <si>
-    <t>30min</t>
-  </si>
-  <si>
-    <t>Correction pour passer de sfml 2 a 3</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="65">
+  <si>
+    <t xml:space="preserve">Matrice de répartition de charges (à remplir à chaque séance)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Séance :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XX/XX/XXXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tâche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etudiant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charge retenue (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commentaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attention :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Seules les tâches techniques sont à inscrire (maths, code, ...).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Les tâches autres (gestion, mise en page, ...) seront valorisées à une charge de 0 heure.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Les tâches réalisées avec une IA doivent faire apparaître IA dans la colonne Etudiant. Elles ne sont pas prises en compte pour la répartition de la charge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. La colonne 'Charge retenue' contient le temps approximatif. Maximum de 2 heures par étudiant et par séance.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. La répartition individuelle est calculée sur la base des heures individuelles retenues et la somme des heures totales retenues.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Cette matrice doit être remplie par le groupe et la répartition indiquée être validée par tout le groupe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Les contributions indiquées doivent refléter l'apport au projet, non le nombre d'heures devant l'écran.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réponse aux questions du 1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration du git</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place du projet avec SFML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1h 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alizee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correction pour passer de sfml 2 a 3</t>
   </si>
   <si>
     <t xml:space="preserve">30min </t>
   </si>
   <si>
-    <t>Code 1,2 conversion</t>
-  </si>
-  <si>
-    <t>Code 1,2 debug</t>
-  </si>
-  <si>
-    <t>1h</t>
-  </si>
-  <si>
-    <t>Formule 1,2</t>
-  </si>
-  <si>
-    <t>Questions 1.2</t>
-  </si>
-  <si>
-    <t>30 min</t>
-  </si>
-  <si>
-    <t>déplacement v1 simple</t>
-  </si>
-  <si>
-    <t>Alizée</t>
-  </si>
-  <si>
-    <t>code et question correspondante</t>
-  </si>
-  <si>
-    <t>déplacement v2 diagonal</t>
+    <t xml:space="preserve">Code 1,2 conversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code 1,2 debug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formule 1,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Questions 1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">déplacement v1 simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alizée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">code et question correspondante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">déplacement v2 diagonal</t>
   </si>
   <si>
     <t xml:space="preserve">Alizée </t>
   </si>
   <si>
-    <t>code et questions correspondantes</t>
-  </si>
-  <si>
-    <t>2.1 Questions 1 à 3</t>
-  </si>
-  <si>
-    <t>Audrey / Elven</t>
-  </si>
-  <si>
-    <t>2.3</t>
-  </si>
-  <si>
-    <t>45min</t>
-  </si>
-  <si>
-    <t>Calcul de la vitesse et affichage en debug, ajout d’un txt pour la police d’écriture et debut question</t>
-  </si>
-  <si>
-    <t>Réglage de problèmes de débug et release</t>
-  </si>
-  <si>
-    <t>2.1 Question 4</t>
-  </si>
-  <si>
-    <t>15 min</t>
-  </si>
-  <si>
-    <t>Le exel contenant la comparaison des résultats se trouve dans le git et est nommé "Courbes_exercices.xlsx"</t>
-  </si>
-  <si>
-    <t>2.2 Équation différentielles question 1 à 3</t>
-  </si>
-  <si>
-    <t>Séances :</t>
-  </si>
-  <si>
-    <t>2.2 Équation différentielles question 4 à 6</t>
-  </si>
-  <si>
-    <t>1h30</t>
+    <t xml:space="preserve">code et questions correspondantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Questions 1 à 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Audrey / Elven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calcul de la vitesse et affichage en debug, ajout d’un txt pour la police d’écriture et debut question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réglage de problèmes de débug et release</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Question 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le exel contenant la comparaison des résultats se trouve dans le git et est nommé "Courbes_exercices.xlsx"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 Équation différentielles question 1 à 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Séances :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 Équation différentielles question 4 à 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1h30</t>
   </si>
   <si>
     <t xml:space="preserve">2.3 fin des calculs et courbes </t>
   </si>
   <si>
-    <t>5 début affichage image</t>
-  </si>
-  <si>
-    <t>Fin affichage image et rotation</t>
-  </si>
-  <si>
-    <t>Aide ia pour le sprite qui etait de taille 0*0 avec une texture de la bonne taille</t>
-  </si>
-  <si>
-    <t>6.1 Ajout d’autres entités</t>
-  </si>
-  <si>
-    <t>aide IA pour la structuration de la classe abstraîte Entity puis modification et restructurationdu code pour le débugage</t>
-  </si>
-  <si>
-    <t>2h</t>
-  </si>
-  <si>
-    <t>5 ajout cadre et rebond</t>
-  </si>
-  <si>
-    <t>5 modification rebond et energie</t>
-  </si>
-  <si>
-    <t>refactorisation debug</t>
+    <t xml:space="preserve">5 début affichage image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fin affichage image et rotation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aide ia pour le sprite qui etait de taille 0*0 avec une texture de la bonne taille</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.1 Ajout d’autres entités</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aide IA pour la structuration de la classe abstraîte Entity puis modification et restructurationdu code pour le débugage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 ajout cadre et rebond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 modification rebond et energie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refactorisation debug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">correction des erreurs liées a la fusion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alizée / Elven </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aide refactoring </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
-      <u/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <u val="single"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -264,7 +289,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -272,46 +297,82 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="New Office">
       <a:dk1>
@@ -353,14 +414,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri Light" pitchFamily="0" charset="1"/>
+        <a:ea typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:cs typeface="Arial" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Arial"/>
-        <a:cs typeface="Arial"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:ea typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:cs typeface="Arial" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -390,7 +451,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -414,7 +475,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -474,46 +535,47 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G83"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G88"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="9.109375" customWidth="1"/>
-    <col min="2" max="2" width="24.21875" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" customWidth="1"/>
-    <col min="5" max="5" width="31.88671875" customWidth="1"/>
-    <col min="6" max="8" width="9.109375" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="31.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="9.11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="0" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
@@ -527,77 +589,77 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="G7" s="4"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="4"/>
       <c r="G8" s="4"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B12" t="s">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="0" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="0" t="s">
         <v>9</v>
       </c>
       <c r="G13" s="4"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B14" t="s">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0" t="s">
         <v>10</v>
       </c>
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="B16" t="s">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B17" t="s">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B18" t="s">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="0" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="5" t="n">
         <v>46274</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="s">
         <v>3</v>
       </c>
@@ -611,7 +673,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="7" t="s">
         <v>15</v>
       </c>
@@ -623,7 +685,7 @@
       </c>
       <c r="E23" s="7"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="7" t="s">
         <v>18</v>
       </c>
@@ -635,7 +697,7 @@
       </c>
       <c r="E24" s="7"/>
     </row>
-    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
         <v>21</v>
       </c>
@@ -647,7 +709,7 @@
       </c>
       <c r="E25" s="7"/>
     </row>
-    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="7" t="s">
         <v>15</v>
       </c>
@@ -659,30 +721,30 @@
       </c>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B30" s="5">
+      <c r="B30" s="5" t="n">
         <v>46275</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="2" t="s">
         <v>3</v>
       </c>
@@ -696,7 +758,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="7" t="s">
         <v>25</v>
       </c>
@@ -708,7 +770,7 @@
       </c>
       <c r="E33" s="7"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="7" t="s">
         <v>27</v>
       </c>
@@ -720,7 +782,7 @@
       </c>
       <c r="E34" s="7"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="7" t="s">
         <v>28</v>
       </c>
@@ -732,7 +794,7 @@
       </c>
       <c r="E35" s="7"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="7" t="s">
         <v>30</v>
       </c>
@@ -744,7 +806,7 @@
       </c>
       <c r="E36" s="7"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="7" t="s">
         <v>31</v>
       </c>
@@ -755,18 +817,18 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B39" s="5">
+      <c r="B39" s="5" t="n">
         <v>46279</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="2" t="s">
         <v>3</v>
       </c>
@@ -780,7 +842,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="8" t="s">
         <v>33</v>
       </c>
@@ -794,7 +856,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="s">
         <v>36</v>
       </c>
@@ -808,7 +870,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="7" t="s">
         <v>39</v>
       </c>
@@ -820,24 +882,24 @@
       </c>
       <c r="E44" s="7"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
       <c r="E45" s="7"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="5">
+      <c r="B46" s="5" t="n">
         <v>46280</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="2" t="s">
         <v>3</v>
       </c>
@@ -851,7 +913,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="7" t="s">
         <v>41</v>
       </c>
@@ -865,7 +927,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="7" t="s">
         <v>44</v>
       </c>
@@ -877,8 +939,8 @@
       </c>
       <c r="E50" s="7"/>
     </row>
-    <row r="51" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B51" t="s">
+    <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="0" t="s">
         <v>45</v>
       </c>
       <c r="C51" s="7" t="s">
@@ -891,7 +953,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="7" t="s">
         <v>48</v>
       </c>
@@ -903,30 +965,30 @@
       </c>
       <c r="E52" s="7"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B55" s="5">
+      <c r="B55" s="5" t="n">
         <v>46282</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="2" t="s">
         <v>3</v>
       </c>
@@ -940,51 +1002,51 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B58" t="s">
+    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C58" s="0" t="s">
         <v>40</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D58" s="0" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B59" t="s">
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C59" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D59" s="0" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B60" t="s">
+    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C60" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D60" s="0" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B64" s="5">
+      <c r="B64" s="5" t="n">
         <v>46283</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2"/>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="6" t="s">
         <v>3</v>
       </c>
@@ -998,7 +1060,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="7" t="s">
         <v>54</v>
       </c>
@@ -1012,7 +1074,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="68" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="7" t="s">
         <v>56</v>
       </c>
@@ -1026,18 +1088,18 @@
         <v>57</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B70" s="5">
+      <c r="B70" s="5" t="n">
         <v>46286</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2"/>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="6" t="s">
         <v>3</v>
       </c>
@@ -1051,7 +1113,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="7" t="s">
         <v>56</v>
       </c>
@@ -1063,7 +1125,7 @@
       </c>
       <c r="E73" s="7"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="7" t="s">
         <v>59</v>
       </c>
@@ -1075,30 +1137,30 @@
       </c>
       <c r="E74" s="7"/>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="7"/>
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
       <c r="E75" s="7"/>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="7"/>
       <c r="C76" s="7"/>
       <c r="D76" s="7"/>
       <c r="E76" s="7"/>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B77" s="5">
+      <c r="B77" s="5" t="n">
         <v>46287</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2"/>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="6" t="s">
         <v>3</v>
       </c>
@@ -1112,7 +1174,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="7" t="s">
         <v>60</v>
       </c>
@@ -1124,7 +1186,7 @@
       </c>
       <c r="E80" s="7"/>
     </row>
-    <row r="81" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B81" s="7" t="s">
         <v>61</v>
       </c>
@@ -1136,20 +1198,72 @@
       </c>
       <c r="E81" s="7"/>
     </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B82" s="7"/>
       <c r="C82" s="7"/>
       <c r="D82" s="7"/>
       <c r="E82" s="7"/>
     </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B83" s="7"/>
       <c r="C83" s="7"/>
       <c r="D83" s="7"/>
       <c r="E83" s="7"/>
     </row>
+    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="2"/>
+    </row>
+    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B86" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E86" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B87" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C87" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="D87" s="0" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B88" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="C88" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="D88" s="0" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.70069444444444495" right="0.70069444444444495" top="0.75208333333333299" bottom="0.75208333333333299" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.700694444444445" right="0.700694444444445" top="0.752083333333333" bottom="0.752083333333333" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>